<commit_message>
Enhance publication bias diagnostics with marginal/conditional residual funnels, variance-controlled time-lags, and dynamic 2-decimal inline R statistics
</commit_message>
<xml_diff>
--- a/data/1_effect_size_calculation_pipeline/Data Extraction Mate Choice Meta Analysis.xlsx
+++ b/data/1_effect_size_calculation_pipeline/Data Extraction Mate Choice Meta Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardosantos/Documents/Repos/mate_choice_meta/data/1_effect_size_calculation_pipeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69AE60E6-CB2C-A642-A352-6FC7A24281DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADC3ED86-E720-804C-94F0-6EBC606B30CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="-20980" windowWidth="38400" windowHeight="20980" activeTab="1" xr2:uid="{6DC7178C-46B5-0C45-81F9-84CEBBB229E2}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{6DC7178C-46B5-0C45-81F9-84CEBBB229E2}"/>
   </bookViews>
   <sheets>
     <sheet name="MetaData" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="LosiaExtraction" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2816,43 +2817,50 @@
   </cellStyles>
   <dxfs count="60">
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Arial "/>
-        <scheme val="none"/>
-      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="8"/>
+          <bgColor theme="8"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Arial "/>
-        <scheme val="none"/>
-      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFBBC04"/>
+          <bgColor rgb="FFFBBC04"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Arial "/>
-        <scheme val="none"/>
-      </font>
       <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.249977111117893"/>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="8"/>
+          <bgColor theme="8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFBBC04"/>
+          <bgColor rgb="FFFBBC04"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3421,50 +3429,43 @@
       </font>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="8"/>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Arial "/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFBBC04"/>
-          <bgColor rgb="FFFBBC04"/>
-        </patternFill>
-      </fill>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Arial "/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Arial "/>
+        <scheme val="none"/>
+      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="8"/>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFBBC04"/>
-          <bgColor rgb="FFFBBC04"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
+        <patternFill>
+          <bgColor theme="2" tint="-0.249977111117893"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3529,56 +3530,56 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{97E449EB-034C-0E47-8DC7-F9320BB33341}" name="Table6" displayName="Table6" ref="A1:AU77" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{97E449EB-034C-0E47-8DC7-F9320BB33341}" name="Table6" displayName="Table6" ref="A1:AU77" headerRowDxfId="55" dataDxfId="54" totalsRowDxfId="53">
   <autoFilter ref="A1:AU77" xr:uid="{97E449EB-034C-0E47-8DC7-F9320BB33341}"/>
   <tableColumns count="47">
-    <tableColumn id="1" xr3:uid="{DB5D9A59-AAEB-A241-9311-F34A51BD8EF0}" name="identifierExtractor" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{F40B866E-46F9-8C4F-A9B6-6B60A705E1E3}" name="identifierStudyId" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{A9DDC2A6-7318-9642-AA36-10E7149E6EF3}" name="identifierStudyYear" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{71F70EE4-3DC2-E14B-98A2-F9CB5439E463}" name="identifierStudyDoi" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{983513C9-9040-FB40-8C65-4484E4B3B536}" name="taxonomySpecies" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{BBAA3805-EF91-624C-B589-EE7D55FFD1F2}" name="experimentalSpeciesOrigin" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{FCC0D2FD-F140-7441-A700-192BC0C30E37}" name="identifierExperimentId" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{D12E62D0-9D27-384B-9D67-EDAC6174B5A9}" name="experimentalDesignType" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{D3578E14-AC1D-EB4A-A629-334B144DBE93}" name="experimentalModelPairing" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{30F8ADE3-D78B-9C4E-B1B2-487EC300E27E}" name="experimentalTypeCopyingMechanism" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{456C1072-BD92-6046-AE56-EDACA565F226}" name="experimentalTypeStimulus" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{8A586C71-977C-7844-9139-2F6C285E46AC}" name="experimentalTypeChoiceTest" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{1FF3CB09-0300-0A43-AFAC-2496AC977AE6}" name="experimentalTypeTestDescription" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{E1164ED1-691B-1447-B5B0-92611E6290CE}" name="experimentalTypeSex" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{A6B91430-639B-074F-A991-A07B7097027D}" name="experimentalTypeVirgin" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{C0209916-95EE-3A46-B0F4-FC4354EDA45C}" name="experimentalModelAge" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{2011A80D-6A98-6347-9901-A3DD63832D93}" name="effectSizeSourceType" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{7B0D63C2-4EA1-114D-9328-2BA848C50E06}" name="effectSizeSourceDetails" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{E4448D55-9F08-DF4A-A7A5-D6D8F77E3066}" name="effectSizeEstimateType" dataDxfId="31"/>
-    <tableColumn id="20" xr3:uid="{7AD1C83E-03F7-154C-8DCE-072CF8C7877B}" name="effectSizeEstimateValue" dataDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{7E567C9D-622D-E14F-A02D-183AC2502CC1}" name="effectSizeEstimateExtra" dataDxfId="29"/>
-    <tableColumn id="22" xr3:uid="{B6FD3F35-3579-8540-89FD-D6121E134326}" name="effectSizeEstimateNotes" dataDxfId="28"/>
-    <tableColumn id="23" xr3:uid="{FECDE26C-A644-BB45-B07B-58D6D1FDF917}" name="effectSizeDirection" dataDxfId="27"/>
-    <tableColumn id="24" xr3:uid="{1C6BD9AE-A05E-8F46-805E-FC9E65560EC0}" name="effectSizeSampleSizeA" dataDxfId="26"/>
-    <tableColumn id="25" xr3:uid="{098FF7F3-2728-DF48-9A4D-3E3995B1420D}" name="effectSizeSampleSizeB" dataDxfId="25"/>
-    <tableColumn id="26" xr3:uid="{68134223-B2A4-744A-9068-78FCB2D1F840}" name="effectSizeSampleSizeC" dataDxfId="24"/>
-    <tableColumn id="27" xr3:uid="{92D0969F-F5FF-E643-95D8-4AA914243C69}" name="effectSizeSampleSizeD" dataDxfId="23"/>
-    <tableColumn id="28" xr3:uid="{391F399A-2B1F-2F45-84E6-E65F91272C76}" name="effectSizesampleSize" dataDxfId="22"/>
-    <tableColumn id="29" xr3:uid="{96BE3409-663C-4E41-950B-277A677EF1BC}" name="controlMean" dataDxfId="21"/>
-    <tableColumn id="30" xr3:uid="{9F830133-B182-5845-855D-21DA97A63F13}" name="controlSD" dataDxfId="20"/>
-    <tableColumn id="31" xr3:uid="{34FAF2C4-428D-4149-841E-24F8F6A19073}" name="controlSE" dataDxfId="19"/>
-    <tableColumn id="32" xr3:uid="{5DF58CF2-4231-0644-8D1D-5B7851A64541}" name="controlN" dataDxfId="18"/>
-    <tableColumn id="33" xr3:uid="{61469D33-0E11-9B45-AE40-48F3597A92EE}" name="treatmentMean" dataDxfId="17"/>
-    <tableColumn id="34" xr3:uid="{C996DB96-1DBC-2941-A0C8-C83106BFA00B}" name="treatmentSD" dataDxfId="16"/>
-    <tableColumn id="35" xr3:uid="{6D30952A-39C6-CB45-9B51-92FBBF4AC74B}" name="treatmentSE" dataDxfId="15"/>
-    <tableColumn id="36" xr3:uid="{8BBE60D8-9BAD-EB46-A6A4-B31BBF9214B9}" name="treatmentN" dataDxfId="14"/>
-    <tableColumn id="37" xr3:uid="{C2A38E50-B1D9-E440-9959-49C758AF57BB}" name="descritionStudyComplexity" dataDxfId="13"/>
-    <tableColumn id="38" xr3:uid="{181FADB4-A9B4-BC46-8DDB-A2C03D5EB80E}" name="effectSizeDataTypeForCalculation" dataDxfId="12"/>
-    <tableColumn id="39" xr3:uid="{912EAD23-33F6-CC41-99AA-9AB5E2FB2DEB}" name="descriptionGeneralNote" dataDxfId="11"/>
-    <tableColumn id="40" xr3:uid="{149F3A48-6134-FF48-8E5B-4390548C0792}" name="effectSizeCalculatedHedgesD" dataDxfId="10"/>
-    <tableColumn id="41" xr3:uid="{D64669C0-6087-3D47-9901-D4632AD62568}" name="effectSizeCalculatedHedgesDVariance" dataDxfId="9"/>
-    <tableColumn id="42" xr3:uid="{388D146B-3E15-0642-8620-4E552753577E}" name="effectSizeHedgesDHowCalculated" dataDxfId="8"/>
-    <tableColumn id="43" xr3:uid="{0D5DC710-67D6-1242-A7A9-033C089D485D}" name="effectSizeCalculatedOddsRatio" dataDxfId="7"/>
-    <tableColumn id="44" xr3:uid="{C9B76442-8E07-4F4A-866A-8A565B70D9D5}" name="effectSizeCalculatedOddsRatioVariance" dataDxfId="6"/>
-    <tableColumn id="45" xr3:uid="{DD14C7AC-EB07-E544-9977-3A24579E917E}" name="effectSizeOddsRatioHowCalculated" dataDxfId="5"/>
-    <tableColumn id="46" xr3:uid="{F3B7075C-9FCA-8C4F-8187-C518F6F97E31}" name="InformationCheckedColumnsFilled" dataDxfId="4"/>
-    <tableColumn id="47" xr3:uid="{82025493-9A53-1E4C-B7D5-3743518D0DBB}" name="RemoveFromDataset" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{DB5D9A59-AAEB-A241-9311-F34A51BD8EF0}" name="identifierExtractor" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{F40B866E-46F9-8C4F-A9B6-6B60A705E1E3}" name="identifierStudyId" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{A9DDC2A6-7318-9642-AA36-10E7149E6EF3}" name="identifierStudyYear" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{71F70EE4-3DC2-E14B-98A2-F9CB5439E463}" name="identifierStudyDoi" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{983513C9-9040-FB40-8C65-4484E4B3B536}" name="taxonomySpecies" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{BBAA3805-EF91-624C-B589-EE7D55FFD1F2}" name="experimentalSpeciesOrigin" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{FCC0D2FD-F140-7441-A700-192BC0C30E37}" name="identifierExperimentId" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{D12E62D0-9D27-384B-9D67-EDAC6174B5A9}" name="experimentalDesignType" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{D3578E14-AC1D-EB4A-A629-334B144DBE93}" name="experimentalModelPairing" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{30F8ADE3-D78B-9C4E-B1B2-487EC300E27E}" name="experimentalTypeCopyingMechanism" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{456C1072-BD92-6046-AE56-EDACA565F226}" name="experimentalTypeStimulus" dataDxfId="42"/>
+    <tableColumn id="12" xr3:uid="{8A586C71-977C-7844-9139-2F6C285E46AC}" name="experimentalTypeChoiceTest" dataDxfId="41"/>
+    <tableColumn id="13" xr3:uid="{1FF3CB09-0300-0A43-AFAC-2496AC977AE6}" name="experimentalTypeTestDescription" dataDxfId="40"/>
+    <tableColumn id="14" xr3:uid="{E1164ED1-691B-1447-B5B0-92611E6290CE}" name="experimentalTypeSex" dataDxfId="39"/>
+    <tableColumn id="15" xr3:uid="{A6B91430-639B-074F-A991-A07B7097027D}" name="experimentalTypeVirgin" dataDxfId="38"/>
+    <tableColumn id="16" xr3:uid="{C0209916-95EE-3A46-B0F4-FC4354EDA45C}" name="experimentalModelAge" dataDxfId="37"/>
+    <tableColumn id="17" xr3:uid="{2011A80D-6A98-6347-9901-A3DD63832D93}" name="effectSizeSourceType" dataDxfId="36"/>
+    <tableColumn id="18" xr3:uid="{7B0D63C2-4EA1-114D-9328-2BA848C50E06}" name="effectSizeSourceDetails" dataDxfId="35"/>
+    <tableColumn id="19" xr3:uid="{E4448D55-9F08-DF4A-A7A5-D6D8F77E3066}" name="effectSizeEstimateType" dataDxfId="34"/>
+    <tableColumn id="20" xr3:uid="{7AD1C83E-03F7-154C-8DCE-072CF8C7877B}" name="effectSizeEstimateValue" dataDxfId="33"/>
+    <tableColumn id="21" xr3:uid="{7E567C9D-622D-E14F-A02D-183AC2502CC1}" name="effectSizeEstimateExtra" dataDxfId="32"/>
+    <tableColumn id="22" xr3:uid="{B6FD3F35-3579-8540-89FD-D6121E134326}" name="effectSizeEstimateNotes" dataDxfId="31"/>
+    <tableColumn id="23" xr3:uid="{FECDE26C-A644-BB45-B07B-58D6D1FDF917}" name="effectSizeDirection" dataDxfId="30"/>
+    <tableColumn id="24" xr3:uid="{1C6BD9AE-A05E-8F46-805E-FC9E65560EC0}" name="effectSizeSampleSizeA" dataDxfId="29"/>
+    <tableColumn id="25" xr3:uid="{098FF7F3-2728-DF48-9A4D-3E3995B1420D}" name="effectSizeSampleSizeB" dataDxfId="28"/>
+    <tableColumn id="26" xr3:uid="{68134223-B2A4-744A-9068-78FCB2D1F840}" name="effectSizeSampleSizeC" dataDxfId="27"/>
+    <tableColumn id="27" xr3:uid="{92D0969F-F5FF-E643-95D8-4AA914243C69}" name="effectSizeSampleSizeD" dataDxfId="26"/>
+    <tableColumn id="28" xr3:uid="{391F399A-2B1F-2F45-84E6-E65F91272C76}" name="effectSizesampleSize" dataDxfId="25"/>
+    <tableColumn id="29" xr3:uid="{96BE3409-663C-4E41-950B-277A677EF1BC}" name="controlMean" dataDxfId="24"/>
+    <tableColumn id="30" xr3:uid="{9F830133-B182-5845-855D-21DA97A63F13}" name="controlSD" dataDxfId="23"/>
+    <tableColumn id="31" xr3:uid="{34FAF2C4-428D-4149-841E-24F8F6A19073}" name="controlSE" dataDxfId="22"/>
+    <tableColumn id="32" xr3:uid="{5DF58CF2-4231-0644-8D1D-5B7851A64541}" name="controlN" dataDxfId="21"/>
+    <tableColumn id="33" xr3:uid="{61469D33-0E11-9B45-AE40-48F3597A92EE}" name="treatmentMean" dataDxfId="20"/>
+    <tableColumn id="34" xr3:uid="{C996DB96-1DBC-2941-A0C8-C83106BFA00B}" name="treatmentSD" dataDxfId="19"/>
+    <tableColumn id="35" xr3:uid="{6D30952A-39C6-CB45-9B51-92FBBF4AC74B}" name="treatmentSE" dataDxfId="18"/>
+    <tableColumn id="36" xr3:uid="{8BBE60D8-9BAD-EB46-A6A4-B31BBF9214B9}" name="treatmentN" dataDxfId="17"/>
+    <tableColumn id="37" xr3:uid="{C2A38E50-B1D9-E440-9959-49C758AF57BB}" name="descritionStudyComplexity" dataDxfId="16"/>
+    <tableColumn id="38" xr3:uid="{181FADB4-A9B4-BC46-8DDB-A2C03D5EB80E}" name="effectSizeDataTypeForCalculation" dataDxfId="15"/>
+    <tableColumn id="39" xr3:uid="{912EAD23-33F6-CC41-99AA-9AB5E2FB2DEB}" name="descriptionGeneralNote" dataDxfId="14"/>
+    <tableColumn id="40" xr3:uid="{149F3A48-6134-FF48-8E5B-4390548C0792}" name="effectSizeCalculatedHedgesD" dataDxfId="13"/>
+    <tableColumn id="41" xr3:uid="{D64669C0-6087-3D47-9901-D4632AD62568}" name="effectSizeCalculatedHedgesDVariance" dataDxfId="12"/>
+    <tableColumn id="42" xr3:uid="{388D146B-3E15-0642-8620-4E552753577E}" name="effectSizeHedgesDHowCalculated" dataDxfId="11"/>
+    <tableColumn id="43" xr3:uid="{0D5DC710-67D6-1242-A7A9-033C089D485D}" name="effectSizeCalculatedOddsRatio" dataDxfId="10"/>
+    <tableColumn id="44" xr3:uid="{C9B76442-8E07-4F4A-866A-8A565B70D9D5}" name="effectSizeCalculatedOddsRatioVariance" dataDxfId="9"/>
+    <tableColumn id="45" xr3:uid="{DD14C7AC-EB07-E544-9977-3A24579E917E}" name="effectSizeOddsRatioHowCalculated" dataDxfId="8"/>
+    <tableColumn id="46" xr3:uid="{F3B7075C-9FCA-8C4F-8187-C518F6F97E31}" name="InformationCheckedColumnsFilled" dataDxfId="7"/>
+    <tableColumn id="47" xr3:uid="{82025493-9A53-1E4C-B7D5-3743518D0DBB}" name="RemoveFromDataset" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="EduardoExtraction-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -14814,24 +14815,24 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="AU2:AU77">
-    <cfRule type="containsText" dxfId="55" priority="4" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH(("Yes"),(AU2))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="5" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH(("No"),(AU2))))</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="53" priority="6">
+    <cfRule type="containsBlanks" dxfId="3" priority="6">
       <formula>LEN(TRIM(AU2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AV2:AV77">
-    <cfRule type="containsText" dxfId="52" priority="1" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH(("Yes"),(AV2))))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="51" priority="2" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH(("No"),(AV2))))</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="50" priority="3">
+    <cfRule type="containsBlanks" dxfId="0" priority="3">
       <formula>LEN(TRIM(AV2))=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Format excluded studies table in portrait, sort alphabetically, sync included studies table, and add PRISMA flowdiagram files
</commit_message>
<xml_diff>
--- a/data/1_effect_size_calculation_pipeline/Data Extraction Mate Choice Meta Analysis.xlsx
+++ b/data/1_effect_size_calculation_pipeline/Data Extraction Mate Choice Meta Analysis.xlsx
@@ -3498,7 +3498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV81"/>
+  <dimension ref="A1:AW81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.28515625" defaultRowHeight="16" customHeight="1"/>
   <cols>
     <col width="9.28515625" customWidth="1" min="1" max="12"/>
@@ -3745,6 +3745,11 @@
       <c r="AV1" s="16" t="inlineStr">
         <is>
           <t>RemoveFromDataset</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>ExclusionReason</t>
         </is>
       </c>
     </row>
@@ -7269,6 +7274,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>Duplicate data (same dataset as Harrison-Weiss_2024)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="14.75" customHeight="1">
       <c r="A20" s="17" t="inlineStr">
@@ -7449,6 +7459,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>Does not contain data to calculate effect sizes</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="14.75" customHeight="1">
       <c r="A21" s="24" t="inlineStr">
@@ -13729,6 +13744,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AW52" t="inlineStr">
+        <is>
+          <t>Does not contain data to calculate effect sizes</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="14.75" customHeight="1">
       <c r="A53" s="24" t="inlineStr">
@@ -13909,6 +13929,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AW53" t="inlineStr">
+        <is>
+          <t>Does not contain data to calculate effect sizes</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="14.75" customHeight="1">
       <c r="A54" s="17" t="inlineStr">
@@ -16557,6 +16582,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AW67" t="inlineStr">
+        <is>
+          <t>Focal subject is male; does not measure female mate-choice copying</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="14.75" customHeight="1">
       <c r="A68" s="17" t="inlineStr">
@@ -16731,6 +16761,11 @@
       <c r="AV68" s="30" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="AW68" t="inlineStr">
+        <is>
+          <t>Does not contain data to calculate effect sizes (only overall GLM F-statistic)</t>
         </is>
       </c>
     </row>
@@ -16817,6 +16852,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AW69" t="inlineStr">
+        <is>
+          <t>Audience effect on male preferences; does not measure female mate-choice copying</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="14.75" customHeight="1">
       <c r="A70" s="17" t="inlineStr">
@@ -17097,6 +17137,11 @@
       <c r="AV71" s="30" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="AW71" t="inlineStr">
+        <is>
+          <t>Study design does not meet inclusion criteria (territorial visit counts, not mate preference)</t>
         </is>
       </c>
     </row>
@@ -18323,6 +18368,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AW78" t="inlineStr">
+        <is>
+          <t>Does not measure mate-choice copying (social learning of mating tactics)</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="14.75" customHeight="1">
       <c r="A79" s="72" t="inlineStr">
@@ -18405,6 +18455,11 @@
       <c r="AV79" s="72" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="AW79" t="inlineStr">
+        <is>
+          <t>Audience effect on male preference concealment; does not measure female mate-choice copying</t>
         </is>
       </c>
     </row>

</xml_diff>